<commit_message>
feat(fase-3a): template + dialog import pesanan
</commit_message>
<xml_diff>
--- a/public/template-import-produk.xlsx
+++ b/public/template-import-produk.xlsx
@@ -6,7 +6,8 @@
     <sheet name="Produk" sheetId="1" r:id="rId1"/>
     <sheet name="StokOpname" sheetId="2" r:id="rId2"/>
     <sheet name="HPP-Update" sheetId="3" r:id="rId3"/>
-    <sheet name="PANDUAN" sheetId="4" r:id="rId4"/>
+    <sheet name="Pesanan" sheetId="4" r:id="rId4"/>
+    <sheet name="PANDUAN" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -634,7 +635,170 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:L4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>NoPesanan*</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Marketplace*</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Tanggal*</v>
+      </c>
+      <c r="D1" t="str">
+        <v>SKU*</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Qty*</v>
+      </c>
+      <c r="F1" t="str">
+        <v>HargaSatuan*</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Buyer</v>
+      </c>
+      <c r="H1" t="str">
+        <v>FeeJenis</v>
+      </c>
+      <c r="I1" t="str">
+        <v>FeeBasis</v>
+      </c>
+      <c r="J1" t="str">
+        <v>FeeNilai</v>
+      </c>
+      <c r="K1" t="str">
+        <v>PPh</v>
+      </c>
+      <c r="L1" t="str">
+        <v>PPN%</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>ORD-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>shopee</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="D2" t="str">
+        <v>BRG-001</v>
+      </c>
+      <c r="E2">
+        <v>2</v>
+      </c>
+      <c r="F2">
+        <v>129000</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Budi</v>
+      </c>
+      <c r="H2" t="str">
+        <v>admin</v>
+      </c>
+      <c r="I2" t="str">
+        <v>persen</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2" t="str">
+        <v>YA</v>
+      </c>
+      <c r="L2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>ORD-001</v>
+      </c>
+      <c r="B3" t="str">
+        <v>shopee</v>
+      </c>
+      <c r="C3" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BRG-002</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>159000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Budi</v>
+      </c>
+      <c r="H3" t="str">
+        <v>admin</v>
+      </c>
+      <c r="I3" t="str">
+        <v>persen</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3" t="str">
+        <v>YA</v>
+      </c>
+      <c r="L3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>ORD-002</v>
+      </c>
+      <c r="B4" t="str">
+        <v>tiktok</v>
+      </c>
+      <c r="C4" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BRG-003</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4">
+        <v>45000</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Siti</v>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v>TIDAK</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -800,9 +964,184 @@
         <v>SKU yang sudah ada = UPDATE (upsert), baru = INSERT.</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Sheet Pesanan (kirim ke /api/order, 2-fase: preview → konfirmasi).</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>NoPesanan*</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Kode pesanan marketplace, dikelompokkan per (Marketplace, NoPesanan)</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Marketplace*</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Bebas (shopee/tiktok/tokopedia/dll), dinormalkan lowercase</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Tanggal*</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Format YYYY-MM-DD valid</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>SKU*</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Harus ada di master produk</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Qty*</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Bilangan bulat &gt;= 1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>HargaSatuan*</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Buyer</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Nama pembeli, bebas</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>FeeJenis</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C26" t="str">
+        <v>admin/service/komisi/ongkir/voucher/affiliate/iklan/lain; kosong = tanpa fee</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>FeeBasis</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C27" t="str">
+        <v>flat/persen, default flat bila FeeJenis diisi</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>FeeNilai</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Bilangan bulat &gt;= 0; persen = % dari (Qty x HargaSatuan)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>PPh</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C29" t="str">
+        <v>YA/TIDAK, default YA</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>PPN%</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Angka &gt;= 0, default 0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v/>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Satu order boleh multi-baris (satu baris = satu SKU).</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Peringatan (tak blokir): order campur baris ber-fee + tanpa-fee.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C33"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(order): import Shopee 2-sheet + bulk fulfill + picklist PDF
- lib/d1/orderImportShopee: gabung sheet orders + Advance Fulfilment
  (qty = orders.Jumlah + jumlah baris Advance; SKU ref -> induk; tolak bila kosong)
- lib/d1/orderTransisi: transisi tunggal + batch atomik (preflight stok agregat,
  satu db.batch, delta dikumpulkan untuk SKU sama); flag stok_dikurangi memisahkan
  status kirim eksternal dari pemotongan stok WMS
- lib/d1/picklist + picklistPdf: agregat per SKU master, PDF A4 dengan kolom cek
- app/api/order: preview-shopee, konfirmasi-shopee, transisi-batch, picklist-pdf
- app/order: checkbox seleksi, toolbar bulk, Picklist PDF, dialog import 2 sheet
- migrasi 0009: kolom stok_dikurangi + no_resi (applied remote)
- template: sheet orders + Advance Fulfilment (format export Shopee)
- test: merge 4, transisi 18, picklist 5; e2e order 7
</commit_message>
<xml_diff>
--- a/public/template-import-produk.xlsx
+++ b/public/template-import-produk.xlsx
@@ -7,7 +7,9 @@
     <sheet name="StokOpname" sheetId="2" r:id="rId2"/>
     <sheet name="HPP-Update" sheetId="3" r:id="rId3"/>
     <sheet name="Pesanan" sheetId="4" r:id="rId4"/>
-    <sheet name="PANDUAN" sheetId="5" r:id="rId5"/>
+    <sheet name="orders" sheetId="5" r:id="rId5"/>
+    <sheet name="Advance Fulfilment" sheetId="6" r:id="rId6"/>
+    <sheet name="PANDUAN" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -798,7 +800,311 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:T3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>No. Pesanan</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Status Pesanan</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Status Pembatalan/ Pengembalian</v>
+      </c>
+      <c r="D1" t="str">
+        <v>No. Resi</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Waktu Pesanan Dibuat</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Metode Pembayaran</v>
+      </c>
+      <c r="G1" t="str">
+        <v>SKU Induk</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Nama Produk</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Nomor Referensi SKU</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Nama Variasi</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Harga Awal</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Harga Setelah Diskon</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Jumlah</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Returned quantity</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Subtotal Pesanan</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Diskon Dari Penjual</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Voucher Ditanggung Penjual</v>
+      </c>
+      <c r="R1" t="str">
+        <v>Paket Diskon (Diskon dari Penjual)</v>
+      </c>
+      <c r="S1" t="str">
+        <v>Username (Pembeli)</v>
+      </c>
+      <c r="T1" t="str">
+        <v>Waktu Pesanan Selesai</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>261010AAA1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Perlu Dikirim</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-10-10 09:15</v>
+      </c>
+      <c r="F2" t="str">
+        <v>COD (Bayar di Tempat)</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Lunch Box TRI J 4in1</v>
+      </c>
+      <c r="I2" t="str">
+        <v>001916</v>
+      </c>
+      <c r="J2" t="str">
+        <v>PINK</v>
+      </c>
+      <c r="K2" t="str">
+        <v>20.000</v>
+      </c>
+      <c r="L2" t="str">
+        <v>18.232</v>
+      </c>
+      <c r="M2" t="str">
+        <v>1</v>
+      </c>
+      <c r="N2" t="str">
+        <v>0</v>
+      </c>
+      <c r="O2" t="str">
+        <v>18.232</v>
+      </c>
+      <c r="P2" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>0</v>
+      </c>
+      <c r="R2" t="str">
+        <v>0</v>
+      </c>
+      <c r="S2" t="str">
+        <v>buyer1</v>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>261010AAA2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Telah Dikirim</v>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>SPXID0000000001A</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-10-10 10:02</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Online Payment</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>Pisau Set Dapur 3in1</v>
+      </c>
+      <c r="I3" t="str">
+        <v>100331</v>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v>10.999</v>
+      </c>
+      <c r="L3" t="str">
+        <v>10.879</v>
+      </c>
+      <c r="M3" t="str">
+        <v>1</v>
+      </c>
+      <c r="N3" t="str">
+        <v>0</v>
+      </c>
+      <c r="O3" t="str">
+        <v>10.879</v>
+      </c>
+      <c r="P3" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>0</v>
+      </c>
+      <c r="R3" t="str">
+        <v>0</v>
+      </c>
+      <c r="S3" t="str">
+        <v>buyer2</v>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:T3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:J3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Booking SN</v>
+      </c>
+      <c r="B1" t="str">
+        <v>No. Resi</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Opsi Pengiriman</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Booking Creation Date</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Waktu Pembayaran Dilakukan</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Nama Produk</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Nomor Referensi SKU</v>
+      </c>
+      <c r="H1" t="str">
+        <v>SKU Induk</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Nama Variasi</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Alamat Pengiriman</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>261010AAA1</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v>SPX Hemat</v>
+      </c>
+      <c r="D2" t="str">
+        <v>2026-10-10 09:16</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-10-10 09:15</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Lunch Box TRI J 4in1</v>
+      </c>
+      <c r="G2" t="str">
+        <v>001916</v>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
+        <v>PINK</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Jl. Contoh No.1, KOTA BANDUNG JAWA BARAT</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>261010AAA1</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>SPX Hemat</v>
+      </c>
+      <c r="D3" t="str">
+        <v>2026-10-10 09:16</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-10-10 09:15</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Lunch Box TRI J 4in1</v>
+      </c>
+      <c r="G3" t="str">
+        <v>001916</v>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>BIRU</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Jl. Contoh No.1, KOTA BANDUNG JAWA BARAT</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C43"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1139,9 +1445,107 @@
         <v>Peringatan (tak blokir): order campur baris ber-fee + tanpa-fee.</v>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v/>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Sheet orders + Advance Fulfilment (format export Shopee).</v>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>No. Pesanan</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C36" t="str">
+        <v>ID order Shopee (satu order boleh multi-baris)</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Nomor Referensi SKU</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Ya*</v>
+      </c>
+      <c r="C37" t="str">
+        <v>SKU master; kosong = pakai SKU Induk</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Jumlah</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Qty baris orders; ditambah jumlah baris Advance untuk SKU sama</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>No. Resi</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Terisi = wajib review: sudah/belum diserahkan ke ekspedisi</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Booking SN</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Sama dengan No. Pesanan; setiap baris Advance bernilai qty 1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Status internal selalu masuk 'pending' (atau 'kirim' bila resi ditandai sudah diserahkan).</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Import TIDAK mengubah stok; pemotongan stok hanya saat aksi Pack.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C33"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(stok): kolom Gudang per baris di import produk
- Kolom Gudang opsional: kosong = gudang pilihan dialog (perilaku lama)
- Terisi = id gudang terdaftar+aktif; tolak per baris bila belum terdaftar
- Dedup per (SKU, Gudang): satu SKU boleh multi-baris beda gudang
- Confirm tulis stock_by_bin + movement restock per gudang; scope admin per baris
- Template: kolom Gudang + contoh multi-gudang + panduan
</commit_message>
<xml_diff>
--- a/public/template-import-produk.xlsx
+++ b/public/template-import-produk.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,24 +422,27 @@
         <v>StokAwal</v>
       </c>
       <c r="F1" t="str">
+        <v>Gudang</v>
+      </c>
+      <c r="G1" t="str">
         <v>HPP</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>HargaJual</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>RakBin</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>StokMin</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Barcode</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Expired(YYYY-MM-DD)</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Aktif</v>
       </c>
     </row>
@@ -459,34 +462,37 @@
       <c r="E2">
         <v>100</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="str">
+        <v>ONLINE</v>
+      </c>
+      <c r="G2">
         <v>75000</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>129000</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>A-01</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>10</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v>8991234567890</v>
       </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
       <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
         <v>YA</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BRG-002</v>
+        <v>BRG-001</v>
       </c>
       <c r="B3" t="str">
-        <v>Celana Chino Slim</v>
+        <v>Kemeja Lengan Panjang</v>
       </c>
       <c r="C3" t="str">
         <v>Pakaian</v>
@@ -495,71 +501,118 @@
         <v>pcs</v>
       </c>
       <c r="E3">
-        <v>50</v>
-      </c>
-      <c r="F3">
-        <v>95000</v>
+        <v>20</v>
+      </c>
+      <c r="F3" t="str">
+        <v>GUDANG-A</v>
       </c>
       <c r="G3">
-        <v>159000</v>
-      </c>
-      <c r="H3" t="str">
-        <v>A-02</v>
-      </c>
-      <c r="I3">
-        <v>5</v>
-      </c>
-      <c r="J3" t="str">
-        <v/>
+        <v>75000</v>
+      </c>
+      <c r="H3">
+        <v>129000</v>
+      </c>
+      <c r="I3" t="str">
+        <v>A-01</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>8991234567890</v>
       </c>
       <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
         <v>YA</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BRG-003</v>
+        <v>BRG-002</v>
       </c>
       <c r="B4" t="str">
-        <v>Kopi Bubuk 250g</v>
+        <v>Celana Chino Slim</v>
       </c>
       <c r="C4" t="str">
-        <v>Makanan</v>
+        <v>Pakaian</v>
       </c>
       <c r="D4" t="str">
         <v>pcs</v>
       </c>
       <c r="E4">
+        <v>50</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4">
+        <v>95000</v>
+      </c>
+      <c r="H4">
+        <v>159000</v>
+      </c>
+      <c r="I4" t="str">
+        <v>A-02</v>
+      </c>
+      <c r="J4">
+        <v>5</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v>YA</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>BRG-003</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Kopi Bubuk 250g</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Makanan</v>
+      </c>
+      <c r="D5" t="str">
+        <v>pcs</v>
+      </c>
+      <c r="E5">
         <v>200</v>
       </c>
-      <c r="F4">
+      <c r="F5" t="str">
+        <v>ONLINE</v>
+      </c>
+      <c r="G5">
         <v>28000</v>
       </c>
-      <c r="G4">
+      <c r="H5">
         <v>45000</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I5" t="str">
         <v>B-01</v>
       </c>
-      <c r="I4">
+      <c r="J5">
         <v>20</v>
       </c>
-      <c r="J4" t="str">
-        <v/>
-      </c>
-      <c r="K4" t="str">
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
         <v>2027-12-31</v>
       </c>
-      <c r="L4" t="str">
+      <c r="M5" t="str">
         <v>YA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1104,7 +1157,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C44"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1169,23 +1222,23 @@
         <v>Tidak</v>
       </c>
       <c r="C6" t="str">
-        <v>Bilangan bulat &gt;= 0, default 0</v>
+        <v>Bilangan bulat &gt;= 0, default 0. Ditulis ke gudang kolom Gudang.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>HPP</v>
+        <v>Gudang</v>
       </c>
       <c r="B7" t="str">
         <v>Tidak</v>
       </c>
       <c r="C7" t="str">
-        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
+        <v>ID gudang terdaftar (huruf besar). Kosong = gudang pilihan saat import. Satu SKU boleh multi-baris untuk gudang berbeda. Gudang belum terdaftar = baris ditolak.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>HargaJual</v>
+        <v>HPP</v>
       </c>
       <c r="B8" t="str">
         <v>Tidak</v>
@@ -1196,94 +1249,94 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>RakBin</v>
+        <v>HargaJual</v>
       </c>
       <c r="B9" t="str">
         <v>Tidak</v>
       </c>
       <c r="C9" t="str">
-        <v>Kode rak/bin, dicatat (bin penuh Fase 2 lanjutan)</v>
+        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>StokMin</v>
+        <v>RakBin</v>
       </c>
       <c r="B10" t="str">
         <v>Tidak</v>
       </c>
       <c r="C10" t="str">
-        <v>Reorder point, default kosong</v>
+        <v>Kode rak/bin, dicatat (bin penuh Fase 2 lanjutan)</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Barcode</v>
+        <v>StokMin</v>
       </c>
       <c r="B11" t="str">
         <v>Tidak</v>
       </c>
       <c r="C11" t="str">
-        <v>Harus unik bila diisi</v>
+        <v>Reorder point, default kosong</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Expired</v>
+        <v>Barcode</v>
       </c>
       <c r="B12" t="str">
         <v>Tidak</v>
       </c>
       <c r="C12" t="str">
-        <v>Format YYYY-MM-DD atau kosong</v>
+        <v>Harus unik bila diisi</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Aktif</v>
+        <v>Expired</v>
       </c>
       <c r="B13" t="str">
         <v>Tidak</v>
       </c>
       <c r="C13" t="str">
-        <v>YA/TIDAK, default YA</v>
+        <v>Format YYYY-MM-DD atau kosong</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v/>
+        <v>Aktif</v>
       </c>
       <c r="B14" t="str">
-        <v/>
+        <v>Tidak</v>
       </c>
       <c r="C14" t="str">
-        <v/>
+        <v>YA/TIDAK, default YA</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Alur import: upload → preview sukses/gagal per baris → Konfirmasi → tulis atomik.</v>
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SKU yang sudah ada = UPDATE (upsert), baru = INSERT.</v>
+        <v>Alur import: upload → preview sukses/gagal per baris → Konfirmasi → tulis atomik.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v/>
-      </c>
-      <c r="B17" t="str">
-        <v/>
-      </c>
-      <c r="C17" t="str">
-        <v/>
+        <v>SKU yang sudah ada = UPDATE (upsert), baru = INSERT.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Sheet Pesanan (kirim ke /api/order, 2-fase: preview → konfirmasi).</v>
+        <v/>
       </c>
       <c r="B18" t="str">
         <v/>
@@ -1294,171 +1347,171 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>NoPesanan*</v>
+        <v>Sheet Pesanan (kirim ke /api/order, 2-fase: preview → konfirmasi).</v>
       </c>
       <c r="B19" t="str">
-        <v>Ya</v>
+        <v/>
       </c>
       <c r="C19" t="str">
-        <v>Kode pesanan marketplace, dikelompokkan per (Marketplace, NoPesanan)</v>
+        <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Marketplace*</v>
+        <v>NoPesanan*</v>
       </c>
       <c r="B20" t="str">
         <v>Ya</v>
       </c>
       <c r="C20" t="str">
-        <v>Bebas (shopee/tiktok/tokopedia/dll), dinormalkan lowercase</v>
+        <v>Kode pesanan marketplace, dikelompokkan per (Marketplace, NoPesanan)</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Tanggal*</v>
+        <v>Marketplace*</v>
       </c>
       <c r="B21" t="str">
         <v>Ya</v>
       </c>
       <c r="C21" t="str">
-        <v>Format YYYY-MM-DD valid</v>
+        <v>Bebas (shopee/tiktok/tokopedia/dll), dinormalkan lowercase</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SKU*</v>
+        <v>Tanggal*</v>
       </c>
       <c r="B22" t="str">
         <v>Ya</v>
       </c>
       <c r="C22" t="str">
-        <v>Harus ada di master produk</v>
+        <v>Format YYYY-MM-DD valid</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Qty*</v>
+        <v>SKU*</v>
       </c>
       <c r="B23" t="str">
         <v>Ya</v>
       </c>
       <c r="C23" t="str">
-        <v>Bilangan bulat &gt;= 1</v>
+        <v>Harus ada di master produk</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>HargaSatuan*</v>
+        <v>Qty*</v>
       </c>
       <c r="B24" t="str">
         <v>Ya</v>
       </c>
       <c r="C24" t="str">
-        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
+        <v>Bilangan bulat &gt;= 1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Buyer</v>
+        <v>HargaSatuan*</v>
       </c>
       <c r="B25" t="str">
-        <v>Tidak</v>
+        <v>Ya</v>
       </c>
       <c r="C25" t="str">
-        <v>Nama pembeli, bebas</v>
+        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>FeeJenis</v>
+        <v>Buyer</v>
       </c>
       <c r="B26" t="str">
         <v>Tidak</v>
       </c>
       <c r="C26" t="str">
-        <v>admin/service/komisi/ongkir/voucher/affiliate/iklan/lain; kosong = tanpa fee</v>
+        <v>Nama pembeli, bebas</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>FeeBasis</v>
+        <v>FeeJenis</v>
       </c>
       <c r="B27" t="str">
         <v>Tidak</v>
       </c>
       <c r="C27" t="str">
-        <v>flat/persen, default flat bila FeeJenis diisi</v>
+        <v>admin/service/komisi/ongkir/voucher/affiliate/iklan/lain; kosong = tanpa fee</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FeeNilai</v>
+        <v>FeeBasis</v>
       </c>
       <c r="B28" t="str">
         <v>Tidak</v>
       </c>
       <c r="C28" t="str">
-        <v>Bilangan bulat &gt;= 0; persen = % dari (Qty x HargaSatuan)</v>
+        <v>flat/persen, default flat bila FeeJenis diisi</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>PPh</v>
+        <v>FeeNilai</v>
       </c>
       <c r="B29" t="str">
         <v>Tidak</v>
       </c>
       <c r="C29" t="str">
-        <v>YA/TIDAK, default YA</v>
+        <v>Bilangan bulat &gt;= 0; persen = % dari (Qty x HargaSatuan)</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>PPN%</v>
+        <v>PPh</v>
       </c>
       <c r="B30" t="str">
         <v>Tidak</v>
       </c>
       <c r="C30" t="str">
-        <v>Angka &gt;= 0, default 0</v>
+        <v>YA/TIDAK, default YA</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v/>
+        <v>PPN%</v>
       </c>
       <c r="B31" t="str">
-        <v/>
+        <v>Tidak</v>
       </c>
       <c r="C31" t="str">
-        <v/>
+        <v>Angka &gt;= 0, default 0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Satu order boleh multi-baris (satu baris = satu SKU).</v>
+        <v/>
+      </c>
+      <c r="B32" t="str">
+        <v/>
+      </c>
+      <c r="C32" t="str">
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Peringatan (tak blokir): order campur baris ber-fee + tanpa-fee.</v>
+        <v>Satu order boleh multi-baris (satu baris = satu SKU).</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v/>
-      </c>
-      <c r="B34" t="str">
-        <v/>
-      </c>
-      <c r="C34" t="str">
-        <v/>
+        <v>Peringatan (tak blokir): order campur baris ber-fee + tanpa-fee.</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Sheet orders + Advance Fulfilment (format export Shopee).</v>
+        <v/>
       </c>
       <c r="B35" t="str">
         <v/>
@@ -1469,83 +1522,94 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>No. Pesanan</v>
+        <v>Sheet orders + Advance Fulfilment (format export Shopee).</v>
       </c>
       <c r="B36" t="str">
-        <v>Ya</v>
+        <v/>
       </c>
       <c r="C36" t="str">
-        <v>ID order Shopee (satu order boleh multi-baris)</v>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Nomor Referensi SKU</v>
+        <v>No. Pesanan</v>
       </c>
       <c r="B37" t="str">
-        <v>Ya*</v>
+        <v>Ya</v>
       </c>
       <c r="C37" t="str">
-        <v>SKU master; kosong = pakai SKU Induk</v>
+        <v>ID order Shopee (satu order boleh multi-baris)</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Jumlah</v>
+        <v>Nomor Referensi SKU</v>
       </c>
       <c r="B38" t="str">
-        <v>Ya</v>
+        <v>Ya*</v>
       </c>
       <c r="C38" t="str">
-        <v>Qty baris orders; ditambah jumlah baris Advance untuk SKU sama</v>
+        <v>SKU master; kosong = pakai SKU Induk</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>No. Resi</v>
+        <v>Jumlah</v>
       </c>
       <c r="B39" t="str">
-        <v>Tidak</v>
+        <v>Ya</v>
       </c>
       <c r="C39" t="str">
-        <v>Terisi = wajib review: sudah/belum diserahkan ke ekspedisi</v>
+        <v>Qty baris orders; ditambah jumlah baris Advance untuk SKU sama</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Booking SN</v>
+        <v>No. Resi</v>
       </c>
       <c r="B40" t="str">
-        <v>Ya</v>
+        <v>Tidak</v>
       </c>
       <c r="C40" t="str">
-        <v>Sama dengan No. Pesanan; setiap baris Advance bernilai qty 1</v>
+        <v>Terisi = wajib review: sudah/belum diserahkan ke ekspedisi</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v/>
+        <v>Booking SN</v>
       </c>
       <c r="B41" t="str">
-        <v/>
+        <v>Ya</v>
       </c>
       <c r="C41" t="str">
-        <v/>
+        <v>Sama dengan No. Pesanan; setiap baris Advance bernilai qty 1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Status internal selalu masuk 'pending' (atau 'kirim' bila resi ditandai sudah diserahkan).</v>
+        <v/>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
+        <v>Status internal selalu masuk 'pending' (atau 'kirim' bila resi ditandai sudah diserahkan).</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
         <v>Import TIDAK mengubah stok; pemotongan stok hanya saat aksi Pack.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C44"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(laba): isi kategori 482 SKU dari export Shopee + konverter EN-ID + template kolom baru + skrip uji nyata
</commit_message>
<xml_diff>
--- a/public/template-import-produk.xlsx
+++ b/public/template-import-produk.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:P4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,203 +416,198 @@
         <v>Kategori</v>
       </c>
       <c r="D1" t="str">
+        <v>Tier Override</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Pre-Order</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Ukuran Khusus</v>
+      </c>
+      <c r="G1" t="str">
         <v>Satuan*</v>
       </c>
-      <c r="E1" t="str">
+      <c r="H1" t="str">
         <v>StokAwal</v>
       </c>
-      <c r="F1" t="str">
+      <c r="I1" t="str">
         <v>Gudang</v>
       </c>
-      <c r="G1" t="str">
+      <c r="J1" t="str">
         <v>HPP</v>
       </c>
-      <c r="H1" t="str">
+      <c r="K1" t="str">
         <v>HargaJual</v>
       </c>
-      <c r="I1" t="str">
+      <c r="L1" t="str">
         <v>RakBin</v>
       </c>
-      <c r="J1" t="str">
+      <c r="M1" t="str">
         <v>StokMin</v>
       </c>
-      <c r="K1" t="str">
+      <c r="N1" t="str">
         <v>Barcode</v>
       </c>
-      <c r="L1" t="str">
+      <c r="O1" t="str">
         <v>Expired(YYYY-MM-DD)</v>
       </c>
-      <c r="M1" t="str">
+      <c r="P1" t="str">
         <v>Aktif</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>BRG-001</v>
+        <v>001916</v>
       </c>
       <c r="B2" t="str">
-        <v>Kemeja Lengan Panjang</v>
+        <v>Lunch Box TRI J 4in1</v>
       </c>
       <c r="C2" t="str">
-        <v>Pakaian</v>
+        <v>Perlengkapan Rumah &gt; Peralatan Makan</v>
       </c>
       <c r="D2" t="str">
+        <v/>
+      </c>
+      <c r="E2" t="str">
+        <v>tidak</v>
+      </c>
+      <c r="F2" t="str">
+        <v>tidak</v>
+      </c>
+      <c r="G2" t="str">
         <v>pcs</v>
       </c>
-      <c r="E2">
+      <c r="H2">
         <v>100</v>
       </c>
-      <c r="F2" t="str">
+      <c r="I2" t="str">
         <v>ONLINE</v>
       </c>
-      <c r="G2">
-        <v>75000</v>
-      </c>
-      <c r="H2">
-        <v>129000</v>
-      </c>
-      <c r="I2" t="str">
+      <c r="J2">
+        <v>15000</v>
+      </c>
+      <c r="K2">
+        <v>18232</v>
+      </c>
+      <c r="L2" t="str">
         <v>A-01</v>
       </c>
-      <c r="J2">
+      <c r="M2">
         <v>10</v>
       </c>
-      <c r="K2" t="str">
-        <v>8991234567890</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
-      </c>
-      <c r="M2" t="str">
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
         <v>YA</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>BRG-001</v>
+        <v>100289</v>
       </c>
       <c r="B3" t="str">
-        <v>Kemeja Lengan Panjang</v>
+        <v>TATAKAN KOMPOR 007</v>
       </c>
       <c r="C3" t="str">
-        <v>Pakaian</v>
+        <v>Elektronik &gt; Perangkat Dapur</v>
       </c>
       <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v>tidak</v>
+      </c>
+      <c r="F3" t="str">
+        <v>tidak</v>
+      </c>
+      <c r="G3" t="str">
         <v>pcs</v>
       </c>
-      <c r="E3">
-        <v>20</v>
-      </c>
-      <c r="F3" t="str">
-        <v>GUDANG-A</v>
-      </c>
-      <c r="G3">
-        <v>75000</v>
-      </c>
       <c r="H3">
-        <v>129000</v>
+        <v>50</v>
       </c>
       <c r="I3" t="str">
-        <v>A-01</v>
+        <v>ONLINE</v>
       </c>
       <c r="J3">
-        <v>10</v>
-      </c>
-      <c r="K3" t="str">
-        <v>8991234567890</v>
+        <v>20000</v>
+      </c>
+      <c r="K3">
+        <v>35000</v>
       </c>
       <c r="L3" t="str">
-        <v/>
-      </c>
-      <c r="M3" t="str">
+        <v>A-02</v>
+      </c>
+      <c r="M3">
+        <v>5</v>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
         <v>YA</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>BRG-002</v>
+        <v>100203</v>
       </c>
       <c r="B4" t="str">
-        <v>Celana Chino Slim</v>
+        <v>Lemari Gantung</v>
       </c>
       <c r="C4" t="str">
-        <v>Pakaian</v>
+        <v>Perlengkapan Rumah &gt; Furniture</v>
       </c>
       <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>tidak</v>
+      </c>
+      <c r="F4" t="str">
+        <v>tidak</v>
+      </c>
+      <c r="G4" t="str">
         <v>pcs</v>
       </c>
-      <c r="E4">
-        <v>50</v>
-      </c>
-      <c r="F4" t="str">
-        <v/>
-      </c>
-      <c r="G4">
-        <v>95000</v>
-      </c>
       <c r="H4">
-        <v>159000</v>
+        <v>20</v>
       </c>
       <c r="I4" t="str">
-        <v>A-02</v>
+        <v>ONLINE</v>
       </c>
       <c r="J4">
+        <v>120000</v>
+      </c>
+      <c r="K4">
+        <v>165000</v>
+      </c>
+      <c r="L4" t="str">
+        <v>B-01</v>
+      </c>
+      <c r="M4">
         <v>5</v>
       </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
-      <c r="L4" t="str">
-        <v/>
-      </c>
-      <c r="M4" t="str">
-        <v>YA</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>BRG-003</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Kopi Bubuk 250g</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Makanan</v>
-      </c>
-      <c r="D5" t="str">
-        <v>pcs</v>
-      </c>
-      <c r="E5">
-        <v>200</v>
-      </c>
-      <c r="F5" t="str">
-        <v>ONLINE</v>
-      </c>
-      <c r="G5">
-        <v>28000</v>
-      </c>
-      <c r="H5">
-        <v>45000</v>
-      </c>
-      <c r="I5" t="str">
-        <v>B-01</v>
-      </c>
-      <c r="J5">
-        <v>20</v>
-      </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
-        <v>2027-12-31</v>
-      </c>
-      <c r="M5" t="str">
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v/>
+      </c>
+      <c r="P4" t="str">
         <v>YA</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1157,7 +1152,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C47"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1200,138 +1195,150 @@
         <v>Tidak</v>
       </c>
       <c r="C4" t="str">
-        <v>Bebas, untuk filter</v>
+        <v>Path Shopee persis spt kategori_tarif (cth: Perlengkapan Rumah &gt; Peralatan Makan). Salah = baris ditolak. Kosong = belum terpetakan + TIDAK menimpa lama.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Satuan*</v>
+        <v>Tier Override</v>
       </c>
       <c r="B5" t="str">
-        <v>Ya</v>
+        <v>Tidak</v>
       </c>
       <c r="C5" t="str">
-        <v>pcs/dus/pak/dll</v>
+        <v>Salah satu tier T10/T9_5/T9/T8_25/T6_75/T6_5/T5_25/T4_25/T2_5. Salah = baris ditolak. Kosong = tidak diubah.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>StokAwal</v>
+        <v>Pre-Order</v>
       </c>
       <c r="B6" t="str">
         <v>Tidak</v>
       </c>
       <c r="C6" t="str">
-        <v>Bilangan bulat &gt;= 0, default 0. Ditulis ke gudang kolom Gudang.</v>
+        <v>ya/tidak (default tidak). Kosong = tidak diubah.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Gudang</v>
+        <v>Ukuran Khusus</v>
       </c>
       <c r="B7" t="str">
         <v>Tidak</v>
       </c>
       <c r="C7" t="str">
-        <v>ID gudang terdaftar (huruf besar). Kosong = gudang pilihan saat import. Satu SKU boleh multi-baris untuk gudang berbeda. Gudang belum terdaftar = baris ditolak.</v>
+        <v>ya/tidak (default tidak; plafon GO XTRA khusus 60rb). Kosong = tidak diubah.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>HPP</v>
+        <v>Satuan*</v>
       </c>
       <c r="B8" t="str">
-        <v>Tidak</v>
+        <v>Ya</v>
       </c>
       <c r="C8" t="str">
-        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
+        <v>pcs/dus/pak/dll</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>HargaJual</v>
+        <v>StokAwal</v>
       </c>
       <c r="B9" t="str">
         <v>Tidak</v>
       </c>
       <c r="C9" t="str">
-        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
+        <v>Bilangan bulat &gt;= 0, default 0. Ditulis ke gudang kolom Gudang.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>RakBin</v>
+        <v>Gudang</v>
       </c>
       <c r="B10" t="str">
         <v>Tidak</v>
       </c>
       <c r="C10" t="str">
-        <v>Kode rak/bin, dicatat (bin penuh Fase 2 lanjutan)</v>
+        <v>ID gudang terdaftar (huruf besar). Kosong = gudang pilihan saat import. Satu SKU boleh multi-baris untuk gudang berbeda. Gudang belum terdaftar = baris ditolak.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>StokMin</v>
+        <v>HPP</v>
       </c>
       <c r="B11" t="str">
         <v>Tidak</v>
       </c>
       <c r="C11" t="str">
-        <v>Reorder point, default kosong</v>
+        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Barcode</v>
+        <v>HargaJual</v>
       </c>
       <c r="B12" t="str">
         <v>Tidak</v>
       </c>
       <c r="C12" t="str">
-        <v>Harus unik bila diisi</v>
+        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Expired</v>
+        <v>RakBin</v>
       </c>
       <c r="B13" t="str">
         <v>Tidak</v>
       </c>
       <c r="C13" t="str">
-        <v>Format YYYY-MM-DD atau kosong</v>
+        <v>Kode rak/bin, dicatat (bin penuh Fase 2 lanjutan)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Aktif</v>
+        <v>StokMin</v>
       </c>
       <c r="B14" t="str">
         <v>Tidak</v>
       </c>
       <c r="C14" t="str">
-        <v>YA/TIDAK, default YA</v>
+        <v>Reorder point, default kosong</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v/>
+        <v>Barcode</v>
       </c>
       <c r="B15" t="str">
-        <v/>
+        <v>Tidak</v>
       </c>
       <c r="C15" t="str">
-        <v/>
+        <v>Harus unik bila diisi</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Alur import: upload → preview sukses/gagal per baris → Konfirmasi → tulis atomik.</v>
+        <v>Expired</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Format YYYY-MM-DD atau kosong</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SKU yang sudah ada = UPDATE (upsert), baru = INSERT.</v>
+        <v>Aktif</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C17" t="str">
+        <v>YA/TIDAK, default YA</v>
       </c>
     </row>
     <row r="18">
@@ -1347,166 +1354,166 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Sheet Pesanan (kirim ke /api/order, 2-fase: preview → konfirmasi).</v>
-      </c>
-      <c r="B19" t="str">
-        <v/>
-      </c>
-      <c r="C19" t="str">
-        <v/>
+        <v>Alur import: upload → preview sukses/gagal per baris → Konfirmasi → tulis atomik.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NoPesanan*</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Ya</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Kode pesanan marketplace, dikelompokkan per (Marketplace, NoPesanan)</v>
+        <v>SKU yang sudah ada = UPDATE (upsert), baru = INSERT.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Marketplace*</v>
+        <v/>
       </c>
       <c r="B21" t="str">
-        <v>Ya</v>
+        <v/>
       </c>
       <c r="C21" t="str">
-        <v>Bebas (shopee/tiktok/tokopedia/dll), dinormalkan lowercase</v>
+        <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Tanggal*</v>
+        <v>Sheet Pesanan (kirim ke /api/order, 2-fase: preview → konfirmasi).</v>
       </c>
       <c r="B22" t="str">
-        <v>Ya</v>
+        <v/>
       </c>
       <c r="C22" t="str">
-        <v>Format YYYY-MM-DD valid</v>
+        <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SKU*</v>
+        <v>NoPesanan*</v>
       </c>
       <c r="B23" t="str">
         <v>Ya</v>
       </c>
       <c r="C23" t="str">
-        <v>Harus ada di master produk</v>
+        <v>Kode pesanan marketplace, dikelompokkan per (Marketplace, NoPesanan)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Qty*</v>
+        <v>Marketplace*</v>
       </c>
       <c r="B24" t="str">
         <v>Ya</v>
       </c>
       <c r="C24" t="str">
-        <v>Bilangan bulat &gt;= 1</v>
+        <v>Bebas (shopee/tiktok/tokopedia/dll), dinormalkan lowercase</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>HargaSatuan*</v>
+        <v>Tanggal*</v>
       </c>
       <c r="B25" t="str">
         <v>Ya</v>
       </c>
       <c r="C25" t="str">
-        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
+        <v>Format YYYY-MM-DD valid</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Buyer</v>
+        <v>SKU*</v>
       </c>
       <c r="B26" t="str">
-        <v>Tidak</v>
+        <v>Ya</v>
       </c>
       <c r="C26" t="str">
-        <v>Nama pembeli, bebas</v>
+        <v>Harus ada di master produk</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>FeeJenis</v>
+        <v>Qty*</v>
       </c>
       <c r="B27" t="str">
-        <v>Tidak</v>
+        <v>Ya</v>
       </c>
       <c r="C27" t="str">
-        <v>admin/service/komisi/ongkir/voucher/affiliate/iklan/lain; kosong = tanpa fee</v>
+        <v>Bilangan bulat &gt;= 1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>FeeBasis</v>
+        <v>HargaSatuan*</v>
       </c>
       <c r="B28" t="str">
-        <v>Tidak</v>
+        <v>Ya</v>
       </c>
       <c r="C28" t="str">
-        <v>flat/persen, default flat bila FeeJenis diisi</v>
+        <v>Bilangan bulat &gt;= 0 (rupiah)</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>FeeNilai</v>
+        <v>Buyer</v>
       </c>
       <c r="B29" t="str">
         <v>Tidak</v>
       </c>
       <c r="C29" t="str">
-        <v>Bilangan bulat &gt;= 0; persen = % dari (Qty x HargaSatuan)</v>
+        <v>Nama pembeli, bebas</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>PPh</v>
+        <v>FeeJenis</v>
       </c>
       <c r="B30" t="str">
         <v>Tidak</v>
       </c>
       <c r="C30" t="str">
-        <v>YA/TIDAK, default YA</v>
+        <v>admin/service/komisi/ongkir/voucher/affiliate/iklan/lain; kosong = tanpa fee</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>PPN%</v>
+        <v>FeeBasis</v>
       </c>
       <c r="B31" t="str">
         <v>Tidak</v>
       </c>
       <c r="C31" t="str">
-        <v>Angka &gt;= 0, default 0</v>
+        <v>flat/persen, default flat bila FeeJenis diisi</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v/>
+        <v>FeeNilai</v>
       </c>
       <c r="B32" t="str">
-        <v/>
+        <v>Tidak</v>
       </c>
       <c r="C32" t="str">
-        <v/>
+        <v>Bilangan bulat &gt;= 0; persen = % dari (Qty x HargaSatuan)</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Satu order boleh multi-baris (satu baris = satu SKU).</v>
+        <v>PPh</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C33" t="str">
+        <v>YA/TIDAK, default YA</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Peringatan (tak blokir): order campur baris ber-fee + tanpa-fee.</v>
+        <v>PPN%</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Angka &gt;= 0, default 0</v>
       </c>
     </row>
     <row r="35">
@@ -1522,94 +1529,115 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Sheet orders + Advance Fulfilment (format export Shopee).</v>
-      </c>
-      <c r="B36" t="str">
-        <v/>
-      </c>
-      <c r="C36" t="str">
-        <v/>
+        <v>Satu order boleh multi-baris (satu baris = satu SKU).</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>No. Pesanan</v>
-      </c>
-      <c r="B37" t="str">
-        <v>Ya</v>
-      </c>
-      <c r="C37" t="str">
-        <v>ID order Shopee (satu order boleh multi-baris)</v>
+        <v>Peringatan (tak blokir): order campur baris ber-fee + tanpa-fee.</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Nomor Referensi SKU</v>
+        <v/>
       </c>
       <c r="B38" t="str">
-        <v>Ya*</v>
+        <v/>
       </c>
       <c r="C38" t="str">
-        <v>SKU master; kosong = pakai SKU Induk</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Jumlah</v>
+        <v>Sheet orders + Advance Fulfilment (format export Shopee).</v>
       </c>
       <c r="B39" t="str">
-        <v>Ya</v>
+        <v/>
       </c>
       <c r="C39" t="str">
-        <v>Qty baris orders; ditambah jumlah baris Advance untuk SKU sama</v>
+        <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>No. Resi</v>
+        <v>No. Pesanan</v>
       </c>
       <c r="B40" t="str">
-        <v>Tidak</v>
+        <v>Ya</v>
       </c>
       <c r="C40" t="str">
-        <v>Terisi = wajib review: sudah/belum diserahkan ke ekspedisi</v>
+        <v>ID order Shopee (satu order boleh multi-baris)</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Booking SN</v>
+        <v>Nomor Referensi SKU</v>
       </c>
       <c r="B41" t="str">
-        <v>Ya</v>
+        <v>Ya*</v>
       </c>
       <c r="C41" t="str">
-        <v>Sama dengan No. Pesanan; setiap baris Advance bernilai qty 1</v>
+        <v>SKU master; kosong = pakai SKU Induk</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v/>
+        <v>Jumlah</v>
       </c>
       <c r="B42" t="str">
-        <v/>
+        <v>Ya</v>
       </c>
       <c r="C42" t="str">
-        <v/>
+        <v>Qty baris orders; ditambah jumlah baris Advance untuk SKU sama</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Status internal selalu masuk 'pending' (atau 'kirim' bila resi ditandai sudah diserahkan).</v>
+        <v>No. Resi</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Tidak</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Terisi = wajib review: sudah/belum diserahkan ke ekspedisi</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
+        <v>Booking SN</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Ya</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Sama dengan No. Pesanan; setiap baris Advance bernilai qty 1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v/>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Status internal selalu masuk 'pending' (atau 'kirim' bila resi ditandai sudah diserahkan).</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
         <v>Import TIDAK mengubah stok; pemotongan stok hanya saat aksi Pack.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C47"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>